<commit_message>
📊 Actualizar CONSULTA_VENTA_VU.xlsx — 01-04-2026, 10:36:48 a. m.
</commit_message>
<xml_diff>
--- a/datos/CONSULTA_VENTA_VU.xlsx
+++ b/datos/CONSULTA_VENTA_VU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{66871571-4161-4DC0-9585-70410936B723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C666ED59-3917-48A1-B172-CEB4635C7452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="459">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -505,18 +505,78 @@
     <t>1015622</t>
   </si>
   <si>
+    <t>22318996-2</t>
+  </si>
+  <si>
+    <t>RODRIGUEZ ESPINOZA ALONSO</t>
+  </si>
+  <si>
+    <t>19/04/1983</t>
+  </si>
+  <si>
     <t>Pedro Aguirre Cerda</t>
   </si>
   <si>
+    <t>5455 - Pedro Aguirre Cerda - Santiago -CP</t>
+  </si>
+  <si>
+    <t>978737691</t>
+  </si>
+  <si>
+    <t>alonsorodriguezespinoza1904@gmail.com; ; ; ;</t>
+  </si>
+  <si>
     <t>11/03/2026</t>
   </si>
   <si>
+    <t>Nf Cartera</t>
+  </si>
+  <si>
     <t>1000000</t>
   </si>
   <si>
+    <t>00/00/0000</t>
+  </si>
+  <si>
     <t>Valle De La Memoria</t>
   </si>
   <si>
+    <t>Valle de la Memoria</t>
+  </si>
+  <si>
+    <t>3-BA-43</t>
+  </si>
+  <si>
+    <t>1015629</t>
+  </si>
+  <si>
+    <t>18190149-7</t>
+  </si>
+  <si>
+    <t>CAYUN HEREDIA KAREN ANDREA</t>
+  </si>
+  <si>
+    <t>03/02/1992</t>
+  </si>
+  <si>
+    <t>Huechuraba</t>
+  </si>
+  <si>
+    <t>228 - Huechuraba - Santiago -CP</t>
+  </si>
+  <si>
+    <t>920512919</t>
+  </si>
+  <si>
+    <t>920234538</t>
+  </si>
+  <si>
+    <t>KARENCAYUNHEREDIA@GMAIL.COM; ; ; ;</t>
+  </si>
+  <si>
+    <t>1347000</t>
+  </si>
+  <si>
     <t>ACTIVO PEND VALIDAR</t>
   </si>
   <si>
@@ -529,6 +589,9 @@
     <t>SIN ASIGNAR</t>
   </si>
   <si>
+    <t>1015631</t>
+  </si>
+  <si>
     <t>10033214-0</t>
   </si>
   <si>
@@ -1040,6 +1103,300 @@
   </si>
   <si>
     <t>1015684</t>
+  </si>
+  <si>
+    <t>10740648-4</t>
+  </si>
+  <si>
+    <t>GALLARDO CONTRERAS SILVIA ISABEL</t>
+  </si>
+  <si>
+    <t>28/10/1967</t>
+  </si>
+  <si>
+    <t>485 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>964469773</t>
+  </si>
+  <si>
+    <t>975782194</t>
+  </si>
+  <si>
+    <t>sigallardo28@hotmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>34.01</t>
+  </si>
+  <si>
+    <t>3880000</t>
+  </si>
+  <si>
+    <t>107778</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>2-AA-4</t>
+  </si>
+  <si>
+    <t>1015686</t>
+  </si>
+  <si>
+    <t>8037977-3</t>
+  </si>
+  <si>
+    <t>ZAMORA MORENO JOSÉ TOMAS</t>
+  </si>
+  <si>
+    <t>28/05/1960</t>
+  </si>
+  <si>
+    <t>548 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>981588402</t>
+  </si>
+  <si>
+    <t>josezamorac.60@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>22/03/2026</t>
+  </si>
+  <si>
+    <t>31/03/2026</t>
+  </si>
+  <si>
+    <t>Ximena Del Carmen Lopez Rozas</t>
+  </si>
+  <si>
+    <t>4100000</t>
+  </si>
+  <si>
+    <t>12.17</t>
+  </si>
+  <si>
+    <t>27/03/2026</t>
+  </si>
+  <si>
+    <t>3601000</t>
+  </si>
+  <si>
+    <t>75021</t>
+  </si>
+  <si>
+    <t>1-AO-16</t>
+  </si>
+  <si>
+    <t>1015697</t>
+  </si>
+  <si>
+    <t>26/03/2026</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>1015701</t>
+  </si>
+  <si>
+    <t>10758714-4</t>
+  </si>
+  <si>
+    <t>VEGA ITURRIETA MARIA MARGARITA</t>
+  </si>
+  <si>
+    <t>27/04/1971</t>
+  </si>
+  <si>
+    <t>158 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>954111244</t>
+  </si>
+  <si>
+    <t>MMVEGA71@GMAIL.COM; ; ; ;</t>
+  </si>
+  <si>
+    <t>29/03/2026</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>1015708</t>
+  </si>
+  <si>
+    <t>18941442-0</t>
+  </si>
+  <si>
+    <t>OLIVARES ACUÑA LORENA ALEXANDRA</t>
+  </si>
+  <si>
+    <t>04/06/1995</t>
+  </si>
+  <si>
+    <t>300 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>946513572</t>
+  </si>
+  <si>
+    <t>lorenaalexandra656@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>3961000</t>
+  </si>
+  <si>
+    <t>397000</t>
+  </si>
+  <si>
+    <t>30/03/2026</t>
+  </si>
+  <si>
+    <t>3564000</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>99000</t>
+  </si>
+  <si>
+    <t>Valle De La Paz</t>
+  </si>
+  <si>
+    <t>Valle de la Paz</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5-Q-69</t>
+  </si>
+  <si>
+    <t>1015711</t>
+  </si>
+  <si>
+    <t>8.944.333-4</t>
+  </si>
+  <si>
+    <t>SOTO LILLO RAMIRO HERNAN</t>
+  </si>
+  <si>
+    <t>04/03/1961</t>
+  </si>
+  <si>
+    <t>730 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>983831323</t>
+  </si>
+  <si>
+    <t>marjorienicole.so@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>21/02/2026</t>
+  </si>
+  <si>
+    <t>3-AI-21</t>
+  </si>
+  <si>
+    <t>1015713</t>
+  </si>
+  <si>
+    <t>7635948-2</t>
+  </si>
+  <si>
+    <t>CID VALDEBENITO JOSÉ ADRIAN</t>
+  </si>
+  <si>
+    <t>26/08/1956</t>
+  </si>
+  <si>
+    <t>12 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>968786800 - 56968786800</t>
+  </si>
+  <si>
+    <t>cidjose547@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>23/03/2026</t>
+  </si>
+  <si>
+    <t>1015714</t>
+  </si>
+  <si>
+    <t>9003503-7</t>
+  </si>
+  <si>
+    <t>MILLA CASTRO HERNAN SERGIO</t>
+  </si>
+  <si>
+    <t>09/10/1960</t>
+  </si>
+  <si>
+    <t>ASENTAMIENTO COLO COLO</t>
+  </si>
+  <si>
+    <t>1620 - ASENTAMIENTO COLO COLO - QUILICURA -CP</t>
+  </si>
+  <si>
+    <t>987779762</t>
+  </si>
+  <si>
+    <t>992530684</t>
+  </si>
+  <si>
+    <t>wally313@hotmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>445000</t>
+  </si>
+  <si>
+    <t>3-I-29</t>
+  </si>
+  <si>
+    <t>1015717</t>
+  </si>
+  <si>
+    <t>20033453-1</t>
+  </si>
+  <si>
+    <t>ROSAS PALOMINOS MARISELA ELIZABETH</t>
+  </si>
+  <si>
+    <t>28/08/1998</t>
+  </si>
+  <si>
+    <t>87 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>994955673</t>
+  </si>
+  <si>
+    <t>rosasmarisela382@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>11.13</t>
+  </si>
+  <si>
+    <t>500000</t>
+  </si>
+  <si>
+    <t>3991000</t>
+  </si>
+  <si>
+    <t>66517</t>
+  </si>
+  <si>
+    <t>4-F-39</t>
+  </si>
+  <si>
+    <t>1015718</t>
   </si>
 </sst>
 </file>
@@ -1900,7 +2257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP21"/>
+  <dimension ref="A1:AP32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="41" width="8" customWidth="1"/>
@@ -2811,58 +3168,58 @@
         <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="D8" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E8" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>164</v>
       </c>
       <c r="G8" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="H8" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="I8" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="J8" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="K8" t="s">
-        <v>176</v>
+        <v>53</v>
       </c>
       <c r="L8" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="M8" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="N8" t="s">
         <v>55</v>
       </c>
       <c r="O8" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="P8" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="Q8" t="s">
-        <v>178</v>
+        <v>65</v>
       </c>
       <c r="R8" t="s">
-        <v>90</v>
+        <v>170</v>
       </c>
       <c r="S8" t="s">
-        <v>91</v>
+        <v>170</v>
       </c>
       <c r="T8" t="s">
-        <v>92</v>
+        <v>170</v>
       </c>
       <c r="U8" t="s">
         <v>60</v>
@@ -2871,31 +3228,31 @@
         <v>60</v>
       </c>
       <c r="W8" t="s">
+        <v>60</v>
+      </c>
+      <c r="X8" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>170</v>
+      </c>
+      <c r="AA8" t="s">
         <v>93</v>
       </c>
-      <c r="X8" t="s">
-        <v>94</v>
-      </c>
-      <c r="Y8" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z8" t="s">
-        <v>95</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>179</v>
-      </c>
       <c r="AB8" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="AC8" t="s">
         <v>67</v>
       </c>
       <c r="AD8" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="AE8" t="s">
-        <v>86</v>
+        <v>172</v>
       </c>
       <c r="AF8" t="s">
         <v>70</v>
@@ -2916,19 +3273,19 @@
         <v>70</v>
       </c>
       <c r="AL8" t="s">
-        <v>49</v>
+        <v>173</v>
       </c>
       <c r="AM8" t="s">
         <v>72</v>
       </c>
       <c r="AN8" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="AO8" t="s">
-        <v>49</v>
+        <v>174</v>
       </c>
       <c r="AP8" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.3">
@@ -2939,34 +3296,34 @@
         <v>43</v>
       </c>
       <c r="C9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D9" t="s">
+        <v>177</v>
+      </c>
+      <c r="E9" t="s">
+        <v>178</v>
+      </c>
+      <c r="F9" t="s">
+        <v>179</v>
+      </c>
+      <c r="G9" t="s">
+        <v>180</v>
+      </c>
+      <c r="H9" t="s">
+        <v>181</v>
+      </c>
+      <c r="I9" t="s">
         <v>182</v>
       </c>
-      <c r="D9" t="s">
+      <c r="J9" t="s">
         <v>183</v>
       </c>
-      <c r="E9" t="s">
-        <v>184</v>
-      </c>
-      <c r="F9" t="s">
-        <v>185</v>
-      </c>
-      <c r="G9" t="s">
-        <v>186</v>
-      </c>
-      <c r="H9" t="s">
-        <v>49</v>
-      </c>
-      <c r="I9" t="s">
-        <v>187</v>
-      </c>
-      <c r="J9" t="s">
-        <v>188</v>
-      </c>
       <c r="K9" t="s">
-        <v>156</v>
+        <v>53</v>
       </c>
       <c r="L9" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="M9" t="s">
         <v>54</v>
@@ -2975,22 +3332,22 @@
         <v>55</v>
       </c>
       <c r="O9" t="s">
-        <v>136</v>
+        <v>49</v>
       </c>
       <c r="P9" t="s">
-        <v>137</v>
+        <v>169</v>
       </c>
       <c r="Q9" t="s">
-        <v>178</v>
+        <v>65</v>
       </c>
       <c r="R9" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="S9" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="T9" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="U9" t="s">
         <v>60</v>
@@ -2999,25 +3356,25 @@
         <v>60</v>
       </c>
       <c r="W9" t="s">
+        <v>60</v>
+      </c>
+      <c r="X9" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>184</v>
+      </c>
+      <c r="AA9" t="s">
         <v>93</v>
       </c>
-      <c r="X9" t="s">
-        <v>190</v>
-      </c>
-      <c r="Y9" t="s">
-        <v>162</v>
-      </c>
-      <c r="Z9" t="s">
-        <v>191</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>192</v>
-      </c>
       <c r="AB9" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="AC9" t="s">
-        <v>67</v>
+        <v>185</v>
       </c>
       <c r="AD9" t="s">
         <v>68</v>
@@ -3044,19 +3401,19 @@
         <v>70</v>
       </c>
       <c r="AL9" t="s">
-        <v>166</v>
+        <v>186</v>
       </c>
       <c r="AM9" t="s">
         <v>72</v>
       </c>
       <c r="AN9" t="s">
-        <v>167</v>
+        <v>187</v>
       </c>
       <c r="AO9" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="AP9" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:42" x14ac:dyDescent="0.3">
@@ -3067,58 +3424,58 @@
         <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="D10" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="E10" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="F10" t="s">
         <v>47</v>
       </c>
       <c r="G10" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="H10" t="s">
-        <v>49</v>
+        <v>194</v>
       </c>
       <c r="I10" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="J10" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="K10" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="L10" t="s">
-        <v>202</v>
+        <v>168</v>
       </c>
       <c r="M10" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="N10" t="s">
         <v>55</v>
       </c>
       <c r="O10" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="P10" t="s">
-        <v>57</v>
+        <v>198</v>
       </c>
       <c r="Q10" t="s">
-        <v>109</v>
+        <v>199</v>
       </c>
       <c r="R10" t="s">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="S10" t="s">
-        <v>139</v>
+        <v>91</v>
       </c>
       <c r="T10" t="s">
-        <v>139</v>
+        <v>92</v>
       </c>
       <c r="U10" t="s">
         <v>60</v>
@@ -3127,31 +3484,31 @@
         <v>60</v>
       </c>
       <c r="W10" t="s">
-        <v>203</v>
+        <v>93</v>
       </c>
       <c r="X10" t="s">
-        <v>204</v>
+        <v>94</v>
       </c>
       <c r="Y10" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="Z10" t="s">
-        <v>205</v>
+        <v>95</v>
       </c>
       <c r="AA10" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="AB10" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="AC10" t="s">
-        <v>165</v>
+        <v>67</v>
       </c>
       <c r="AD10" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="AE10" t="s">
-        <v>164</v>
+        <v>86</v>
       </c>
       <c r="AF10" t="s">
         <v>70</v>
@@ -3172,19 +3529,19 @@
         <v>70</v>
       </c>
       <c r="AL10" t="s">
-        <v>208</v>
+        <v>49</v>
       </c>
       <c r="AM10" t="s">
         <v>72</v>
       </c>
       <c r="AN10" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="AO10" t="s">
-        <v>209</v>
+        <v>49</v>
       </c>
       <c r="AP10" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11" spans="1:42" x14ac:dyDescent="0.3">
@@ -3195,58 +3552,58 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="D11" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="E11" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="F11" t="s">
-        <v>47</v>
+        <v>206</v>
       </c>
       <c r="G11" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="H11" t="s">
-        <v>215</v>
+        <v>49</v>
       </c>
       <c r="I11" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="J11" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="K11" t="s">
-        <v>201</v>
+        <v>156</v>
       </c>
       <c r="L11" t="s">
-        <v>217</v>
+        <v>168</v>
       </c>
       <c r="M11" t="s">
-        <v>218</v>
+        <v>54</v>
       </c>
       <c r="N11" t="s">
         <v>55</v>
       </c>
       <c r="O11" t="s">
-        <v>219</v>
+        <v>136</v>
       </c>
       <c r="P11" t="s">
-        <v>220</v>
+        <v>137</v>
       </c>
       <c r="Q11" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="R11" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="S11" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="T11" t="s">
-        <v>223</v>
+        <v>210</v>
       </c>
       <c r="U11" t="s">
         <v>60</v>
@@ -3255,31 +3612,31 @@
         <v>60</v>
       </c>
       <c r="W11" t="s">
-        <v>224</v>
+        <v>93</v>
       </c>
       <c r="X11" t="s">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="Y11" t="s">
-        <v>226</v>
+        <v>168</v>
       </c>
       <c r="Z11" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="AA11" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="AB11" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="AC11" t="s">
         <v>67</v>
       </c>
       <c r="AD11" t="s">
-        <v>230</v>
+        <v>68</v>
       </c>
       <c r="AE11" t="s">
-        <v>218</v>
+        <v>69</v>
       </c>
       <c r="AF11" t="s">
         <v>70</v>
@@ -3300,19 +3657,19 @@
         <v>70</v>
       </c>
       <c r="AL11" t="s">
-        <v>49</v>
+        <v>186</v>
       </c>
       <c r="AM11" t="s">
         <v>72</v>
       </c>
       <c r="AN11" t="s">
-        <v>49</v>
+        <v>187</v>
       </c>
       <c r="AO11" t="s">
-        <v>49</v>
+        <v>188</v>
       </c>
       <c r="AP11" t="s">
-        <v>231</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" spans="1:42" x14ac:dyDescent="0.3">
@@ -3323,58 +3680,58 @@
         <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>232</v>
+        <v>216</v>
       </c>
       <c r="D12" t="s">
-        <v>233</v>
+        <v>217</v>
       </c>
       <c r="E12" t="s">
-        <v>234</v>
+        <v>218</v>
       </c>
       <c r="F12" t="s">
         <v>47</v>
       </c>
       <c r="G12" t="s">
-        <v>235</v>
+        <v>219</v>
       </c>
       <c r="H12" t="s">
         <v>49</v>
       </c>
       <c r="I12" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="J12" t="s">
-        <v>237</v>
+        <v>221</v>
       </c>
       <c r="K12" t="s">
-        <v>63</v>
+        <v>222</v>
       </c>
       <c r="L12" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="M12" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="N12" t="s">
         <v>55</v>
       </c>
       <c r="O12" t="s">
-        <v>153</v>
+        <v>56</v>
       </c>
       <c r="P12" t="s">
-        <v>238</v>
+        <v>57</v>
       </c>
       <c r="Q12" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="R12" t="s">
-        <v>90</v>
+        <v>139</v>
       </c>
       <c r="S12" t="s">
-        <v>91</v>
+        <v>139</v>
       </c>
       <c r="T12" t="s">
-        <v>92</v>
+        <v>139</v>
       </c>
       <c r="U12" t="s">
         <v>60</v>
@@ -3383,31 +3740,31 @@
         <v>60</v>
       </c>
       <c r="W12" t="s">
-        <v>93</v>
+        <v>224</v>
       </c>
       <c r="X12" t="s">
-        <v>94</v>
+        <v>225</v>
       </c>
       <c r="Y12" t="s">
-        <v>239</v>
+        <v>223</v>
       </c>
       <c r="Z12" t="s">
-        <v>95</v>
+        <v>226</v>
       </c>
       <c r="AA12" t="s">
-        <v>96</v>
+        <v>227</v>
       </c>
       <c r="AB12" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="AC12" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="AD12" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="AE12" t="s">
-        <v>86</v>
+        <v>172</v>
       </c>
       <c r="AF12" t="s">
         <v>70</v>
@@ -3428,19 +3785,19 @@
         <v>70</v>
       </c>
       <c r="AL12" t="s">
-        <v>49</v>
+        <v>229</v>
       </c>
       <c r="AM12" t="s">
         <v>72</v>
       </c>
       <c r="AN12" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="AO12" t="s">
-        <v>49</v>
+        <v>230</v>
       </c>
       <c r="AP12" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:42" x14ac:dyDescent="0.3">
@@ -3451,91 +3808,91 @@
         <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="D13" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="E13" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="F13" t="s">
         <v>47</v>
       </c>
       <c r="G13" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="H13" t="s">
-        <v>49</v>
+        <v>236</v>
       </c>
       <c r="I13" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="J13" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="K13" t="s">
+        <v>222</v>
+      </c>
+      <c r="L13" t="s">
+        <v>238</v>
+      </c>
+      <c r="M13" t="s">
         <v>239</v>
-      </c>
-      <c r="L13" t="s">
-        <v>217</v>
-      </c>
-      <c r="M13" t="s">
-        <v>218</v>
       </c>
       <c r="N13" t="s">
         <v>55</v>
       </c>
       <c r="O13" t="s">
-        <v>153</v>
+        <v>240</v>
       </c>
       <c r="P13" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>199</v>
+      </c>
+      <c r="R13" t="s">
+        <v>242</v>
+      </c>
+      <c r="S13" t="s">
+        <v>243</v>
+      </c>
+      <c r="T13" t="s">
+        <v>244</v>
+      </c>
+      <c r="U13" t="s">
+        <v>60</v>
+      </c>
+      <c r="V13" t="s">
+        <v>60</v>
+      </c>
+      <c r="W13" t="s">
+        <v>245</v>
+      </c>
+      <c r="X13" t="s">
+        <v>246</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>247</v>
+      </c>
+      <c r="Z13" t="s">
         <v>248</v>
       </c>
-      <c r="Q13" t="s">
-        <v>89</v>
-      </c>
-      <c r="R13" t="s">
+      <c r="AA13" t="s">
         <v>249</v>
       </c>
-      <c r="S13" t="s">
+      <c r="AB13" t="s">
         <v>250</v>
-      </c>
-      <c r="T13" t="s">
-        <v>250</v>
-      </c>
-      <c r="U13" t="s">
-        <v>60</v>
-      </c>
-      <c r="V13" t="s">
-        <v>60</v>
-      </c>
-      <c r="W13" t="s">
-        <v>93</v>
-      </c>
-      <c r="X13" t="s">
-        <v>251</v>
-      </c>
-      <c r="Y13" t="s">
-        <v>239</v>
-      </c>
-      <c r="Z13" t="s">
-        <v>252</v>
-      </c>
-      <c r="AA13" t="s">
-        <v>253</v>
-      </c>
-      <c r="AB13" t="s">
-        <v>254</v>
       </c>
       <c r="AC13" t="s">
         <v>67</v>
       </c>
       <c r="AD13" t="s">
-        <v>230</v>
+        <v>251</v>
       </c>
       <c r="AE13" t="s">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="AF13" t="s">
         <v>70</v>
@@ -3568,7 +3925,7 @@
         <v>49</v>
       </c>
       <c r="AP13" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="14" spans="1:42" x14ac:dyDescent="0.3">
@@ -3579,34 +3936,34 @@
         <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D14" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E14" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="F14" t="s">
         <v>47</v>
       </c>
       <c r="G14" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="H14" t="s">
         <v>49</v>
       </c>
       <c r="I14" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J14" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="K14" t="s">
-        <v>107</v>
+        <v>63</v>
       </c>
       <c r="L14" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="M14" t="s">
         <v>86</v>
@@ -3615,13 +3972,13 @@
         <v>55</v>
       </c>
       <c r="O14" t="s">
-        <v>219</v>
+        <v>153</v>
       </c>
       <c r="P14" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="Q14" t="s">
-        <v>178</v>
+        <v>138</v>
       </c>
       <c r="R14" t="s">
         <v>90</v>
@@ -3645,19 +4002,19 @@
         <v>94</v>
       </c>
       <c r="Y14" t="s">
-        <v>217</v>
+        <v>260</v>
       </c>
       <c r="Z14" t="s">
         <v>95</v>
       </c>
       <c r="AA14" t="s">
-        <v>253</v>
+        <v>96</v>
       </c>
       <c r="AB14" t="s">
-        <v>180</v>
+        <v>261</v>
       </c>
       <c r="AC14" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="AD14" t="s">
         <v>98</v>
@@ -3696,7 +4053,7 @@
         <v>49</v>
       </c>
       <c r="AP14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" spans="1:42" x14ac:dyDescent="0.3">
@@ -3707,58 +4064,58 @@
         <v>43</v>
       </c>
       <c r="C15" t="s">
+        <v>263</v>
+      </c>
+      <c r="D15" t="s">
         <v>264</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>265</v>
-      </c>
-      <c r="E15" t="s">
-        <v>266</v>
       </c>
       <c r="F15" t="s">
         <v>47</v>
       </c>
       <c r="G15" t="s">
+        <v>266</v>
+      </c>
+      <c r="H15" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" t="s">
         <v>267</v>
       </c>
-      <c r="H15" t="s">
+      <c r="J15" t="s">
         <v>268</v>
       </c>
-      <c r="I15" t="s">
-        <v>268</v>
-      </c>
-      <c r="J15" t="s">
-        <v>269</v>
-      </c>
       <c r="K15" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="L15" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="M15" t="s">
-        <v>86</v>
+        <v>239</v>
       </c>
       <c r="N15" t="s">
         <v>55</v>
       </c>
       <c r="O15" t="s">
-        <v>87</v>
+        <v>153</v>
       </c>
       <c r="P15" t="s">
-        <v>108</v>
+        <v>269</v>
       </c>
       <c r="Q15" t="s">
-        <v>178</v>
+        <v>89</v>
       </c>
       <c r="R15" t="s">
-        <v>90</v>
+        <v>270</v>
       </c>
       <c r="S15" t="s">
-        <v>91</v>
+        <v>271</v>
       </c>
       <c r="T15" t="s">
-        <v>92</v>
+        <v>271</v>
       </c>
       <c r="U15" t="s">
         <v>60</v>
@@ -3770,28 +4127,28 @@
         <v>93</v>
       </c>
       <c r="X15" t="s">
-        <v>94</v>
+        <v>272</v>
       </c>
       <c r="Y15" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="Z15" t="s">
-        <v>95</v>
+        <v>273</v>
       </c>
       <c r="AA15" t="s">
-        <v>253</v>
+        <v>274</v>
       </c>
       <c r="AB15" t="s">
-        <v>180</v>
+        <v>275</v>
       </c>
       <c r="AC15" t="s">
         <v>67</v>
       </c>
       <c r="AD15" t="s">
-        <v>98</v>
+        <v>251</v>
       </c>
       <c r="AE15" t="s">
-        <v>86</v>
+        <v>239</v>
       </c>
       <c r="AF15" t="s">
         <v>70</v>
@@ -3824,7 +4181,7 @@
         <v>49</v>
       </c>
       <c r="AP15" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="16" spans="1:42" x14ac:dyDescent="0.3">
@@ -3835,58 +4192,58 @@
         <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
       <c r="D16" t="s">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="E16" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="F16" t="s">
         <v>47</v>
       </c>
       <c r="G16" t="s">
-        <v>267</v>
+        <v>280</v>
       </c>
       <c r="H16" t="s">
-        <v>268</v>
+        <v>49</v>
       </c>
       <c r="I16" t="s">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="J16" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
       <c r="K16" t="s">
-        <v>270</v>
+        <v>107</v>
       </c>
       <c r="L16" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="M16" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="N16" t="s">
         <v>55</v>
       </c>
       <c r="O16" t="s">
-        <v>87</v>
+        <v>240</v>
       </c>
       <c r="P16" t="s">
-        <v>108</v>
+        <v>283</v>
       </c>
       <c r="Q16" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="R16" t="s">
-        <v>272</v>
+        <v>90</v>
       </c>
       <c r="S16" t="s">
-        <v>272</v>
+        <v>91</v>
       </c>
       <c r="T16" t="s">
-        <v>272</v>
+        <v>92</v>
       </c>
       <c r="U16" t="s">
         <v>60</v>
@@ -3895,31 +4252,31 @@
         <v>60</v>
       </c>
       <c r="W16" t="s">
-        <v>273</v>
+        <v>93</v>
       </c>
       <c r="X16" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA16" t="s">
         <v>274</v>
       </c>
-      <c r="Y16" t="s">
-        <v>275</v>
-      </c>
-      <c r="Z16" t="s">
-        <v>276</v>
-      </c>
-      <c r="AA16" t="s">
-        <v>253</v>
-      </c>
       <c r="AB16" t="s">
-        <v>277</v>
+        <v>201</v>
       </c>
       <c r="AC16" t="s">
-        <v>67</v>
+        <v>185</v>
       </c>
       <c r="AD16" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="AE16" t="s">
-        <v>278</v>
+        <v>86</v>
       </c>
       <c r="AF16" t="s">
         <v>70</v>
@@ -3940,19 +4297,19 @@
         <v>70</v>
       </c>
       <c r="AL16" t="s">
-        <v>166</v>
+        <v>49</v>
       </c>
       <c r="AM16" t="s">
         <v>72</v>
       </c>
       <c r="AN16" t="s">
-        <v>167</v>
+        <v>49</v>
       </c>
       <c r="AO16" t="s">
-        <v>168</v>
+        <v>49</v>
       </c>
       <c r="AP16" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="17" spans="1:42" x14ac:dyDescent="0.3">
@@ -3963,37 +4320,37 @@
         <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="D17" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="E17" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="F17" t="s">
         <v>47</v>
       </c>
       <c r="G17" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="H17" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="I17" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="J17" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="K17" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="L17" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="M17" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="N17" t="s">
         <v>55</v>
@@ -4002,19 +4359,19 @@
         <v>87</v>
       </c>
       <c r="P17" t="s">
-        <v>287</v>
+        <v>108</v>
       </c>
       <c r="Q17" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="R17" t="s">
-        <v>142</v>
+        <v>90</v>
       </c>
       <c r="S17" t="s">
-        <v>142</v>
+        <v>91</v>
       </c>
       <c r="T17" t="s">
-        <v>142</v>
+        <v>92</v>
       </c>
       <c r="U17" t="s">
         <v>60</v>
@@ -4023,31 +4380,31 @@
         <v>60</v>
       </c>
       <c r="W17" t="s">
-        <v>288</v>
+        <v>93</v>
       </c>
       <c r="X17" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>291</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA17" t="s">
         <v>274</v>
       </c>
-      <c r="Y17" t="s">
-        <v>286</v>
-      </c>
-      <c r="Z17" t="s">
-        <v>289</v>
-      </c>
-      <c r="AA17" t="s">
-        <v>253</v>
-      </c>
       <c r="AB17" t="s">
-        <v>290</v>
+        <v>201</v>
       </c>
       <c r="AC17" t="s">
-        <v>165</v>
+        <v>67</v>
       </c>
       <c r="AD17" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="AE17" t="s">
-        <v>164</v>
+        <v>86</v>
       </c>
       <c r="AF17" t="s">
         <v>70</v>
@@ -4068,19 +4425,19 @@
         <v>70</v>
       </c>
       <c r="AL17" t="s">
-        <v>166</v>
+        <v>49</v>
       </c>
       <c r="AM17" t="s">
         <v>72</v>
       </c>
       <c r="AN17" t="s">
-        <v>167</v>
+        <v>49</v>
       </c>
       <c r="AO17" t="s">
-        <v>168</v>
+        <v>49</v>
       </c>
       <c r="AP17" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="18" spans="1:42" x14ac:dyDescent="0.3">
@@ -4091,58 +4448,58 @@
         <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="D18" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="E18" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="F18" t="s">
-        <v>161</v>
+        <v>47</v>
       </c>
       <c r="G18" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="H18" t="s">
-        <v>49</v>
+        <v>289</v>
       </c>
       <c r="I18" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="J18" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="K18" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="L18" t="s">
-        <v>299</v>
+        <v>238</v>
       </c>
       <c r="M18" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="N18" t="s">
         <v>55</v>
       </c>
       <c r="O18" t="s">
-        <v>153</v>
+        <v>87</v>
       </c>
       <c r="P18" t="s">
-        <v>248</v>
+        <v>108</v>
       </c>
       <c r="Q18" t="s">
-        <v>300</v>
+        <v>199</v>
       </c>
       <c r="R18" t="s">
-        <v>90</v>
+        <v>293</v>
       </c>
       <c r="S18" t="s">
-        <v>91</v>
+        <v>293</v>
       </c>
       <c r="T18" t="s">
-        <v>92</v>
+        <v>293</v>
       </c>
       <c r="U18" t="s">
         <v>60</v>
@@ -4151,31 +4508,31 @@
         <v>60</v>
       </c>
       <c r="W18" t="s">
-        <v>93</v>
+        <v>294</v>
       </c>
       <c r="X18" t="s">
-        <v>94</v>
+        <v>295</v>
       </c>
       <c r="Y18" t="s">
+        <v>296</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>297</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>274</v>
+      </c>
+      <c r="AB18" t="s">
         <v>298</v>
       </c>
-      <c r="Z18" t="s">
-        <v>95</v>
-      </c>
-      <c r="AA18" t="s">
-        <v>96</v>
-      </c>
-      <c r="AB18" t="s">
-        <v>301</v>
-      </c>
       <c r="AC18" t="s">
-        <v>165</v>
+        <v>67</v>
       </c>
       <c r="AD18" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="AE18" t="s">
-        <v>86</v>
+        <v>299</v>
       </c>
       <c r="AF18" t="s">
         <v>70</v>
@@ -4196,19 +4553,19 @@
         <v>70</v>
       </c>
       <c r="AL18" t="s">
-        <v>49</v>
+        <v>186</v>
       </c>
       <c r="AM18" t="s">
         <v>72</v>
       </c>
       <c r="AN18" t="s">
-        <v>49</v>
+        <v>187</v>
       </c>
       <c r="AO18" t="s">
-        <v>49</v>
+        <v>188</v>
       </c>
       <c r="AP18" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="19" spans="1:42" x14ac:dyDescent="0.3">
@@ -4219,34 +4576,34 @@
         <v>43</v>
       </c>
       <c r="C19" t="s">
+        <v>301</v>
+      </c>
+      <c r="D19" t="s">
+        <v>302</v>
+      </c>
+      <c r="E19" t="s">
         <v>303</v>
       </c>
-      <c r="D19" t="s">
+      <c r="F19" t="s">
+        <v>47</v>
+      </c>
+      <c r="G19" t="s">
         <v>304</v>
       </c>
-      <c r="E19" t="s">
+      <c r="H19" t="s">
         <v>305</v>
       </c>
-      <c r="F19" t="s">
+      <c r="I19" t="s">
+        <v>305</v>
+      </c>
+      <c r="J19" t="s">
         <v>306</v>
       </c>
-      <c r="G19" t="s">
+      <c r="K19" t="s">
         <v>307</v>
       </c>
-      <c r="H19" t="s">
-        <v>49</v>
-      </c>
-      <c r="I19" t="s">
-        <v>308</v>
-      </c>
-      <c r="J19" t="s">
-        <v>309</v>
-      </c>
-      <c r="K19" t="s">
-        <v>270</v>
-      </c>
       <c r="L19" t="s">
-        <v>299</v>
+        <v>238</v>
       </c>
       <c r="M19" t="s">
         <v>54</v>
@@ -4255,22 +4612,22 @@
         <v>55</v>
       </c>
       <c r="O19" t="s">
-        <v>219</v>
+        <v>87</v>
       </c>
       <c r="P19" t="s">
-        <v>262</v>
+        <v>308</v>
       </c>
       <c r="Q19" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="R19" t="s">
-        <v>189</v>
+        <v>142</v>
       </c>
       <c r="S19" t="s">
-        <v>189</v>
+        <v>142</v>
       </c>
       <c r="T19" t="s">
-        <v>189</v>
+        <v>142</v>
       </c>
       <c r="U19" t="s">
         <v>60</v>
@@ -4279,31 +4636,31 @@
         <v>60</v>
       </c>
       <c r="W19" t="s">
+        <v>309</v>
+      </c>
+      <c r="X19" t="s">
+        <v>295</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>307</v>
+      </c>
+      <c r="Z19" t="s">
         <v>310</v>
       </c>
-      <c r="X19" t="s">
+      <c r="AA19" t="s">
+        <v>274</v>
+      </c>
+      <c r="AB19" t="s">
         <v>311</v>
       </c>
-      <c r="Y19" t="s">
-        <v>270</v>
-      </c>
-      <c r="Z19" t="s">
-        <v>312</v>
-      </c>
-      <c r="AA19" t="s">
-        <v>143</v>
-      </c>
-      <c r="AB19" t="s">
-        <v>313</v>
-      </c>
       <c r="AC19" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="AD19" t="s">
         <v>68</v>
       </c>
       <c r="AE19" t="s">
-        <v>69</v>
+        <v>172</v>
       </c>
       <c r="AF19" t="s">
         <v>70</v>
@@ -4324,19 +4681,19 @@
         <v>70</v>
       </c>
       <c r="AL19" t="s">
-        <v>314</v>
+        <v>186</v>
       </c>
       <c r="AM19" t="s">
         <v>72</v>
       </c>
       <c r="AN19" t="s">
-        <v>73</v>
+        <v>187</v>
       </c>
       <c r="AO19" t="s">
-        <v>315</v>
+        <v>188</v>
       </c>
       <c r="AP19" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
     </row>
     <row r="20" spans="1:42" x14ac:dyDescent="0.3">
@@ -4347,34 +4704,34 @@
         <v>43</v>
       </c>
       <c r="C20" t="s">
+        <v>313</v>
+      </c>
+      <c r="D20" t="s">
+        <v>314</v>
+      </c>
+      <c r="E20" t="s">
+        <v>315</v>
+      </c>
+      <c r="F20" t="s">
+        <v>164</v>
+      </c>
+      <c r="G20" t="s">
+        <v>316</v>
+      </c>
+      <c r="H20" t="s">
+        <v>49</v>
+      </c>
+      <c r="I20" t="s">
         <v>317</v>
       </c>
-      <c r="D20" t="s">
+      <c r="J20" t="s">
         <v>318</v>
       </c>
-      <c r="E20" t="s">
+      <c r="K20" t="s">
         <v>319</v>
       </c>
-      <c r="F20" t="s">
+      <c r="L20" t="s">
         <v>320</v>
-      </c>
-      <c r="G20" t="s">
-        <v>321</v>
-      </c>
-      <c r="H20" t="s">
-        <v>49</v>
-      </c>
-      <c r="I20" t="s">
-        <v>322</v>
-      </c>
-      <c r="J20" t="s">
-        <v>323</v>
-      </c>
-      <c r="K20" t="s">
-        <v>298</v>
-      </c>
-      <c r="L20" t="s">
-        <v>324</v>
       </c>
       <c r="M20" t="s">
         <v>86</v>
@@ -4386,10 +4743,10 @@
         <v>153</v>
       </c>
       <c r="P20" t="s">
-        <v>325</v>
+        <v>269</v>
       </c>
       <c r="Q20" t="s">
-        <v>300</v>
+        <v>321</v>
       </c>
       <c r="R20" t="s">
         <v>90</v>
@@ -4407,25 +4764,25 @@
         <v>60</v>
       </c>
       <c r="W20" t="s">
-        <v>326</v>
+        <v>93</v>
       </c>
       <c r="X20" t="s">
-        <v>163</v>
+        <v>94</v>
       </c>
       <c r="Y20" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="Z20" t="s">
-        <v>327</v>
+        <v>95</v>
       </c>
       <c r="AA20" t="s">
-        <v>328</v>
+        <v>96</v>
       </c>
       <c r="AB20" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="AC20" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="AD20" t="s">
         <v>98</v>
@@ -4464,7 +4821,7 @@
         <v>49</v>
       </c>
       <c r="AP20" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
     </row>
     <row r="21" spans="1:42" x14ac:dyDescent="0.3">
@@ -4475,58 +4832,58 @@
         <v>43</v>
       </c>
       <c r="C21" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="D21" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="E21" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="F21" t="s">
-        <v>47</v>
+        <v>327</v>
       </c>
       <c r="G21" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="H21" t="s">
-        <v>335</v>
+        <v>49</v>
       </c>
       <c r="I21" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="J21" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="K21" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="L21" t="s">
-        <v>299</v>
+        <v>320</v>
       </c>
       <c r="M21" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="N21" t="s">
         <v>55</v>
       </c>
       <c r="O21" t="s">
-        <v>153</v>
+        <v>240</v>
       </c>
       <c r="P21" t="s">
-        <v>325</v>
+        <v>283</v>
       </c>
       <c r="Q21" t="s">
-        <v>300</v>
+        <v>199</v>
       </c>
       <c r="R21" t="s">
-        <v>90</v>
+        <v>210</v>
       </c>
       <c r="S21" t="s">
-        <v>91</v>
+        <v>210</v>
       </c>
       <c r="T21" t="s">
-        <v>92</v>
+        <v>210</v>
       </c>
       <c r="U21" t="s">
         <v>60</v>
@@ -4535,31 +4892,31 @@
         <v>60</v>
       </c>
       <c r="W21" t="s">
-        <v>93</v>
+        <v>331</v>
       </c>
       <c r="X21" t="s">
-        <v>94</v>
+        <v>332</v>
       </c>
       <c r="Y21" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="Z21" t="s">
-        <v>95</v>
+        <v>333</v>
       </c>
       <c r="AA21" t="s">
-        <v>338</v>
+        <v>143</v>
       </c>
       <c r="AB21" t="s">
-        <v>301</v>
+        <v>334</v>
       </c>
       <c r="AC21" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="AD21" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="AE21" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="AF21" t="s">
         <v>70</v>
@@ -4580,19 +4937,1427 @@
         <v>70</v>
       </c>
       <c r="AL21" t="s">
-        <v>49</v>
+        <v>335</v>
       </c>
       <c r="AM21" t="s">
         <v>72</v>
       </c>
       <c r="AN21" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="AO21" t="s">
-        <v>49</v>
+        <v>336</v>
       </c>
       <c r="AP21" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="22" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" t="s">
+        <v>338</v>
+      </c>
+      <c r="D22" t="s">
         <v>339</v>
+      </c>
+      <c r="E22" t="s">
+        <v>340</v>
+      </c>
+      <c r="F22" t="s">
+        <v>341</v>
+      </c>
+      <c r="G22" t="s">
+        <v>342</v>
+      </c>
+      <c r="H22" t="s">
+        <v>49</v>
+      </c>
+      <c r="I22" t="s">
+        <v>343</v>
+      </c>
+      <c r="J22" t="s">
+        <v>344</v>
+      </c>
+      <c r="K22" t="s">
+        <v>319</v>
+      </c>
+      <c r="L22" t="s">
+        <v>345</v>
+      </c>
+      <c r="M22" t="s">
+        <v>86</v>
+      </c>
+      <c r="N22" t="s">
+        <v>55</v>
+      </c>
+      <c r="O22" t="s">
+        <v>153</v>
+      </c>
+      <c r="P22" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>321</v>
+      </c>
+      <c r="R22" t="s">
+        <v>90</v>
+      </c>
+      <c r="S22" t="s">
+        <v>91</v>
+      </c>
+      <c r="T22" t="s">
+        <v>92</v>
+      </c>
+      <c r="U22" t="s">
+        <v>60</v>
+      </c>
+      <c r="V22" t="s">
+        <v>60</v>
+      </c>
+      <c r="W22" t="s">
+        <v>347</v>
+      </c>
+      <c r="X22" t="s">
+        <v>170</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>345</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>348</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>349</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>350</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH22" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI22" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ22" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK22" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL22" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM22" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN22" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO22" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP22" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="23" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" t="s">
+        <v>352</v>
+      </c>
+      <c r="D23" t="s">
+        <v>353</v>
+      </c>
+      <c r="E23" t="s">
+        <v>354</v>
+      </c>
+      <c r="F23" t="s">
+        <v>47</v>
+      </c>
+      <c r="G23" t="s">
+        <v>355</v>
+      </c>
+      <c r="H23" t="s">
+        <v>356</v>
+      </c>
+      <c r="I23" t="s">
+        <v>357</v>
+      </c>
+      <c r="J23" t="s">
+        <v>358</v>
+      </c>
+      <c r="K23" t="s">
+        <v>320</v>
+      </c>
+      <c r="L23" t="s">
+        <v>320</v>
+      </c>
+      <c r="M23" t="s">
+        <v>86</v>
+      </c>
+      <c r="N23" t="s">
+        <v>55</v>
+      </c>
+      <c r="O23" t="s">
+        <v>153</v>
+      </c>
+      <c r="P23" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>321</v>
+      </c>
+      <c r="R23" t="s">
+        <v>90</v>
+      </c>
+      <c r="S23" t="s">
+        <v>91</v>
+      </c>
+      <c r="T23" t="s">
+        <v>92</v>
+      </c>
+      <c r="U23" t="s">
+        <v>60</v>
+      </c>
+      <c r="V23" t="s">
+        <v>60</v>
+      </c>
+      <c r="W23" t="s">
+        <v>93</v>
+      </c>
+      <c r="X23" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>320</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>359</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>322</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG23" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH23" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI23" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ23" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK23" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL23" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM23" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN23" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO23" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP23" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="24" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" t="s">
+        <v>361</v>
+      </c>
+      <c r="D24" t="s">
+        <v>362</v>
+      </c>
+      <c r="E24" t="s">
+        <v>363</v>
+      </c>
+      <c r="F24" t="s">
+        <v>47</v>
+      </c>
+      <c r="G24" t="s">
+        <v>364</v>
+      </c>
+      <c r="H24" t="s">
+        <v>365</v>
+      </c>
+      <c r="I24" t="s">
+        <v>366</v>
+      </c>
+      <c r="J24" t="s">
+        <v>367</v>
+      </c>
+      <c r="K24" t="s">
+        <v>345</v>
+      </c>
+      <c r="L24" t="s">
+        <v>345</v>
+      </c>
+      <c r="M24" t="s">
+        <v>54</v>
+      </c>
+      <c r="N24" t="s">
+        <v>55</v>
+      </c>
+      <c r="O24" t="s">
+        <v>49</v>
+      </c>
+      <c r="P24" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>199</v>
+      </c>
+      <c r="R24" t="s">
+        <v>210</v>
+      </c>
+      <c r="S24" t="s">
+        <v>210</v>
+      </c>
+      <c r="T24" t="s">
+        <v>210</v>
+      </c>
+      <c r="U24" t="s">
+        <v>60</v>
+      </c>
+      <c r="V24" t="s">
+        <v>60</v>
+      </c>
+      <c r="W24" t="s">
+        <v>368</v>
+      </c>
+      <c r="X24" t="s">
+        <v>348</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>345</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>200</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>370</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>69</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG24" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH24" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI24" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ24" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK24" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL24" t="s">
+        <v>71</v>
+      </c>
+      <c r="AM24" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN24" t="s">
+        <v>371</v>
+      </c>
+      <c r="AO24" t="s">
+        <v>372</v>
+      </c>
+      <c r="AP24" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="25" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>42</v>
+      </c>
+      <c r="B25" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" t="s">
+        <v>374</v>
+      </c>
+      <c r="D25" t="s">
+        <v>375</v>
+      </c>
+      <c r="E25" t="s">
+        <v>376</v>
+      </c>
+      <c r="F25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G25" t="s">
+        <v>377</v>
+      </c>
+      <c r="H25" t="s">
+        <v>49</v>
+      </c>
+      <c r="I25" t="s">
+        <v>378</v>
+      </c>
+      <c r="J25" t="s">
+        <v>379</v>
+      </c>
+      <c r="K25" t="s">
+        <v>380</v>
+      </c>
+      <c r="L25" t="s">
+        <v>381</v>
+      </c>
+      <c r="M25" t="s">
+        <v>54</v>
+      </c>
+      <c r="N25" t="s">
+        <v>55</v>
+      </c>
+      <c r="O25" t="s">
+        <v>136</v>
+      </c>
+      <c r="P25" t="s">
+        <v>382</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>89</v>
+      </c>
+      <c r="R25" t="s">
+        <v>383</v>
+      </c>
+      <c r="S25" t="s">
+        <v>383</v>
+      </c>
+      <c r="T25" t="s">
+        <v>383</v>
+      </c>
+      <c r="U25" t="s">
+        <v>60</v>
+      </c>
+      <c r="V25" t="s">
+        <v>60</v>
+      </c>
+      <c r="W25" t="s">
+        <v>384</v>
+      </c>
+      <c r="X25" t="s">
+        <v>141</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>385</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>386</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>158</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>387</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE25" t="s">
+        <v>69</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG25" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH25" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI25" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ25" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK25" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL25" t="s">
+        <v>335</v>
+      </c>
+      <c r="AM25" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN25" t="s">
+        <v>73</v>
+      </c>
+      <c r="AO25" t="s">
+        <v>388</v>
+      </c>
+      <c r="AP25" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="26" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" t="s">
+        <v>374</v>
+      </c>
+      <c r="D26" t="s">
+        <v>375</v>
+      </c>
+      <c r="E26" t="s">
+        <v>376</v>
+      </c>
+      <c r="F26" t="s">
+        <v>47</v>
+      </c>
+      <c r="G26" t="s">
+        <v>377</v>
+      </c>
+      <c r="H26" t="s">
+        <v>49</v>
+      </c>
+      <c r="I26" t="s">
+        <v>378</v>
+      </c>
+      <c r="J26" t="s">
+        <v>379</v>
+      </c>
+      <c r="K26" t="s">
+        <v>390</v>
+      </c>
+      <c r="L26" t="s">
+        <v>381</v>
+      </c>
+      <c r="M26" t="s">
+        <v>86</v>
+      </c>
+      <c r="N26" t="s">
+        <v>55</v>
+      </c>
+      <c r="O26" t="s">
+        <v>136</v>
+      </c>
+      <c r="P26" t="s">
+        <v>382</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>89</v>
+      </c>
+      <c r="R26" t="s">
+        <v>90</v>
+      </c>
+      <c r="S26" t="s">
+        <v>91</v>
+      </c>
+      <c r="T26" t="s">
+        <v>92</v>
+      </c>
+      <c r="U26" t="s">
+        <v>60</v>
+      </c>
+      <c r="V26" t="s">
+        <v>60</v>
+      </c>
+      <c r="W26" t="s">
+        <v>93</v>
+      </c>
+      <c r="X26" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>385</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA26" t="s">
+        <v>391</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC26" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD26" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE26" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF26" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG26" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH26" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI26" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ26" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK26" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL26" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM26" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN26" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO26" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP26" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="27" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" t="s">
+        <v>393</v>
+      </c>
+      <c r="D27" t="s">
+        <v>394</v>
+      </c>
+      <c r="E27" t="s">
+        <v>395</v>
+      </c>
+      <c r="F27" t="s">
+        <v>47</v>
+      </c>
+      <c r="G27" t="s">
+        <v>396</v>
+      </c>
+      <c r="H27" t="s">
+        <v>49</v>
+      </c>
+      <c r="I27" t="s">
+        <v>397</v>
+      </c>
+      <c r="J27" t="s">
+        <v>398</v>
+      </c>
+      <c r="K27" t="s">
+        <v>156</v>
+      </c>
+      <c r="L27" t="s">
+        <v>381</v>
+      </c>
+      <c r="M27" t="s">
+        <v>86</v>
+      </c>
+      <c r="N27" t="s">
+        <v>55</v>
+      </c>
+      <c r="O27" t="s">
+        <v>240</v>
+      </c>
+      <c r="P27" t="s">
+        <v>283</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>199</v>
+      </c>
+      <c r="R27" t="s">
+        <v>90</v>
+      </c>
+      <c r="S27" t="s">
+        <v>91</v>
+      </c>
+      <c r="T27" t="s">
+        <v>92</v>
+      </c>
+      <c r="U27" t="s">
+        <v>60</v>
+      </c>
+      <c r="V27" t="s">
+        <v>60</v>
+      </c>
+      <c r="W27" t="s">
+        <v>93</v>
+      </c>
+      <c r="X27" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y27" t="s">
+        <v>399</v>
+      </c>
+      <c r="Z27" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA27" t="s">
+        <v>400</v>
+      </c>
+      <c r="AB27" t="s">
+        <v>201</v>
+      </c>
+      <c r="AC27" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD27" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE27" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF27" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG27" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH27" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI27" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ27" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK27" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL27" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM27" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN27" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO27" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP27" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="28" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" t="s">
+        <v>402</v>
+      </c>
+      <c r="D28" t="s">
+        <v>403</v>
+      </c>
+      <c r="E28" t="s">
+        <v>404</v>
+      </c>
+      <c r="F28" t="s">
+        <v>47</v>
+      </c>
+      <c r="G28" t="s">
+        <v>405</v>
+      </c>
+      <c r="H28" t="s">
+        <v>49</v>
+      </c>
+      <c r="I28" t="s">
+        <v>406</v>
+      </c>
+      <c r="J28" t="s">
+        <v>407</v>
+      </c>
+      <c r="K28" t="s">
+        <v>390</v>
+      </c>
+      <c r="L28" t="s">
+        <v>381</v>
+      </c>
+      <c r="M28" t="s">
+        <v>54</v>
+      </c>
+      <c r="N28" t="s">
+        <v>55</v>
+      </c>
+      <c r="O28" t="s">
+        <v>240</v>
+      </c>
+      <c r="P28" t="s">
+        <v>283</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>199</v>
+      </c>
+      <c r="R28" t="s">
+        <v>408</v>
+      </c>
+      <c r="S28" t="s">
+        <v>408</v>
+      </c>
+      <c r="T28" t="s">
+        <v>408</v>
+      </c>
+      <c r="U28" t="s">
+        <v>60</v>
+      </c>
+      <c r="V28" t="s">
+        <v>60</v>
+      </c>
+      <c r="W28" t="s">
+        <v>309</v>
+      </c>
+      <c r="X28" t="s">
+        <v>409</v>
+      </c>
+      <c r="Y28" t="s">
+        <v>410</v>
+      </c>
+      <c r="Z28" t="s">
+        <v>411</v>
+      </c>
+      <c r="AA28" t="s">
+        <v>412</v>
+      </c>
+      <c r="AB28" t="s">
+        <v>413</v>
+      </c>
+      <c r="AC28" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD28" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE28" t="s">
+        <v>414</v>
+      </c>
+      <c r="AF28" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG28" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH28" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI28" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ28" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK28" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL28" t="s">
+        <v>415</v>
+      </c>
+      <c r="AM28" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN28" t="s">
+        <v>416</v>
+      </c>
+      <c r="AO28" t="s">
+        <v>417</v>
+      </c>
+      <c r="AP28" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="29" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" t="s">
+        <v>419</v>
+      </c>
+      <c r="D29" t="s">
+        <v>420</v>
+      </c>
+      <c r="E29" t="s">
+        <v>421</v>
+      </c>
+      <c r="F29" t="s">
+        <v>47</v>
+      </c>
+      <c r="G29" t="s">
+        <v>422</v>
+      </c>
+      <c r="H29" t="s">
+        <v>49</v>
+      </c>
+      <c r="I29" t="s">
+        <v>423</v>
+      </c>
+      <c r="J29" t="s">
+        <v>424</v>
+      </c>
+      <c r="K29" t="s">
+        <v>425</v>
+      </c>
+      <c r="L29" t="s">
+        <v>381</v>
+      </c>
+      <c r="M29" t="s">
+        <v>54</v>
+      </c>
+      <c r="N29" t="s">
+        <v>55</v>
+      </c>
+      <c r="O29" t="s">
+        <v>56</v>
+      </c>
+      <c r="P29" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>138</v>
+      </c>
+      <c r="R29" t="s">
+        <v>139</v>
+      </c>
+      <c r="S29" t="s">
+        <v>139</v>
+      </c>
+      <c r="T29" t="s">
+        <v>139</v>
+      </c>
+      <c r="U29" t="s">
+        <v>60</v>
+      </c>
+      <c r="V29" t="s">
+        <v>60</v>
+      </c>
+      <c r="W29" t="s">
+        <v>140</v>
+      </c>
+      <c r="X29" t="s">
+        <v>141</v>
+      </c>
+      <c r="Y29" t="s">
+        <v>390</v>
+      </c>
+      <c r="Z29" t="s">
+        <v>142</v>
+      </c>
+      <c r="AA29" t="s">
+        <v>96</v>
+      </c>
+      <c r="AB29" t="s">
+        <v>144</v>
+      </c>
+      <c r="AC29" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD29" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE29" t="s">
+        <v>172</v>
+      </c>
+      <c r="AF29" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG29" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH29" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI29" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ29" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK29" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL29" t="s">
+        <v>173</v>
+      </c>
+      <c r="AM29" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN29" t="s">
+        <v>73</v>
+      </c>
+      <c r="AO29" t="s">
+        <v>426</v>
+      </c>
+      <c r="AP29" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="30" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" t="s">
+        <v>428</v>
+      </c>
+      <c r="D30" t="s">
+        <v>429</v>
+      </c>
+      <c r="E30" t="s">
+        <v>430</v>
+      </c>
+      <c r="F30" t="s">
+        <v>47</v>
+      </c>
+      <c r="G30" t="s">
+        <v>431</v>
+      </c>
+      <c r="H30" t="s">
+        <v>49</v>
+      </c>
+      <c r="I30" t="s">
+        <v>432</v>
+      </c>
+      <c r="J30" t="s">
+        <v>433</v>
+      </c>
+      <c r="K30" t="s">
+        <v>434</v>
+      </c>
+      <c r="L30" t="s">
+        <v>381</v>
+      </c>
+      <c r="M30" t="s">
+        <v>86</v>
+      </c>
+      <c r="N30" t="s">
+        <v>55</v>
+      </c>
+      <c r="O30" t="s">
+        <v>136</v>
+      </c>
+      <c r="P30" t="s">
+        <v>382</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>89</v>
+      </c>
+      <c r="R30" t="s">
+        <v>90</v>
+      </c>
+      <c r="S30" t="s">
+        <v>91</v>
+      </c>
+      <c r="T30" t="s">
+        <v>92</v>
+      </c>
+      <c r="U30" t="s">
+        <v>60</v>
+      </c>
+      <c r="V30" t="s">
+        <v>60</v>
+      </c>
+      <c r="W30" t="s">
+        <v>93</v>
+      </c>
+      <c r="X30" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y30" t="s">
+        <v>410</v>
+      </c>
+      <c r="Z30" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA30" t="s">
+        <v>391</v>
+      </c>
+      <c r="AB30" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC30" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD30" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE30" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF30" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG30" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH30" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI30" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ30" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK30" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL30" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM30" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN30" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO30" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP30" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="31" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" t="s">
+        <v>436</v>
+      </c>
+      <c r="D31" t="s">
+        <v>437</v>
+      </c>
+      <c r="E31" t="s">
+        <v>438</v>
+      </c>
+      <c r="F31" t="s">
+        <v>439</v>
+      </c>
+      <c r="G31" t="s">
+        <v>440</v>
+      </c>
+      <c r="H31" t="s">
+        <v>441</v>
+      </c>
+      <c r="I31" t="s">
+        <v>442</v>
+      </c>
+      <c r="J31" t="s">
+        <v>443</v>
+      </c>
+      <c r="K31" t="s">
+        <v>410</v>
+      </c>
+      <c r="L31" t="s">
+        <v>381</v>
+      </c>
+      <c r="M31" t="s">
+        <v>54</v>
+      </c>
+      <c r="N31" t="s">
+        <v>55</v>
+      </c>
+      <c r="O31" t="s">
+        <v>49</v>
+      </c>
+      <c r="P31" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>65</v>
+      </c>
+      <c r="R31" t="s">
+        <v>444</v>
+      </c>
+      <c r="S31" t="s">
+        <v>444</v>
+      </c>
+      <c r="T31" t="s">
+        <v>444</v>
+      </c>
+      <c r="U31" t="s">
+        <v>60</v>
+      </c>
+      <c r="V31" t="s">
+        <v>60</v>
+      </c>
+      <c r="W31" t="s">
+        <v>60</v>
+      </c>
+      <c r="X31" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z31" t="s">
+        <v>444</v>
+      </c>
+      <c r="AA31" t="s">
+        <v>391</v>
+      </c>
+      <c r="AB31" t="s">
+        <v>444</v>
+      </c>
+      <c r="AC31" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD31" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE31" t="s">
+        <v>172</v>
+      </c>
+      <c r="AF31" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG31" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH31" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI31" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ31" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK31" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL31" t="s">
+        <v>173</v>
+      </c>
+      <c r="AM31" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN31" t="s">
+        <v>73</v>
+      </c>
+      <c r="AO31" t="s">
+        <v>445</v>
+      </c>
+      <c r="AP31" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="32" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" t="s">
+        <v>447</v>
+      </c>
+      <c r="D32" t="s">
+        <v>448</v>
+      </c>
+      <c r="E32" t="s">
+        <v>449</v>
+      </c>
+      <c r="F32" t="s">
+        <v>47</v>
+      </c>
+      <c r="G32" t="s">
+        <v>450</v>
+      </c>
+      <c r="H32" t="s">
+        <v>49</v>
+      </c>
+      <c r="I32" t="s">
+        <v>451</v>
+      </c>
+      <c r="J32" t="s">
+        <v>452</v>
+      </c>
+      <c r="K32" t="s">
+        <v>345</v>
+      </c>
+      <c r="L32" t="s">
+        <v>381</v>
+      </c>
+      <c r="M32" t="s">
+        <v>54</v>
+      </c>
+      <c r="N32" t="s">
+        <v>55</v>
+      </c>
+      <c r="O32" t="s">
+        <v>56</v>
+      </c>
+      <c r="P32" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>138</v>
+      </c>
+      <c r="R32" t="s">
+        <v>139</v>
+      </c>
+      <c r="S32" t="s">
+        <v>139</v>
+      </c>
+      <c r="T32" t="s">
+        <v>139</v>
+      </c>
+      <c r="U32" t="s">
+        <v>60</v>
+      </c>
+      <c r="V32" t="s">
+        <v>60</v>
+      </c>
+      <c r="W32" t="s">
+        <v>453</v>
+      </c>
+      <c r="X32" t="s">
+        <v>454</v>
+      </c>
+      <c r="Y32" t="s">
+        <v>390</v>
+      </c>
+      <c r="Z32" t="s">
+        <v>455</v>
+      </c>
+      <c r="AA32" t="s">
+        <v>96</v>
+      </c>
+      <c r="AB32" t="s">
+        <v>456</v>
+      </c>
+      <c r="AC32" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD32" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE32" t="s">
+        <v>172</v>
+      </c>
+      <c r="AF32" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG32" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH32" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI32" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ32" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK32" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL32" t="s">
+        <v>229</v>
+      </c>
+      <c r="AM32" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN32" t="s">
+        <v>416</v>
+      </c>
+      <c r="AO32" t="s">
+        <v>457</v>
+      </c>
+      <c r="AP32" t="s">
+        <v>458</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Actualizar CONSULTA_VENTA_VU.xlsx — 01-04-2026, 3:48:18 p. m.
</commit_message>
<xml_diff>
--- a/datos/CONSULTA_VENTA_VU.xlsx
+++ b/datos/CONSULTA_VENTA_VU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C666ED59-3917-48A1-B172-CEB4635C7452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6AD33DF5-CF8F-49CB-97EF-9E4ED9D08FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1764" uniqueCount="564">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -1397,6 +1397,321 @@
   </si>
   <si>
     <t>1015718</t>
+  </si>
+  <si>
+    <t>8626435-8</t>
+  </si>
+  <si>
+    <t>CARRASCO HERNANDEZ MARTA</t>
+  </si>
+  <si>
+    <t>29/11/1959</t>
+  </si>
+  <si>
+    <t>5838 - Renca - Santiago -CP</t>
+  </si>
+  <si>
+    <t>954940199</t>
+  </si>
+  <si>
+    <t>936883029</t>
+  </si>
+  <si>
+    <t>jessica.carrasco46@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>Andrea Valeska Saffa Romero</t>
+  </si>
+  <si>
+    <t>1015719</t>
+  </si>
+  <si>
+    <t>10068490-K</t>
+  </si>
+  <si>
+    <t>GAETE OSORIO MARINA DE LAS MERCEDES</t>
+  </si>
+  <si>
+    <t>17/05/1964</t>
+  </si>
+  <si>
+    <t>767 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>988987431</t>
+  </si>
+  <si>
+    <t>marna.gaete01@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>28/03/2026</t>
+  </si>
+  <si>
+    <t>01/04/2026</t>
+  </si>
+  <si>
+    <t>1015720</t>
+  </si>
+  <si>
+    <t>17065070-0</t>
+  </si>
+  <si>
+    <t>LOPEZ RUZ ENRIQUE ANTONIO</t>
+  </si>
+  <si>
+    <t>17/01/1989</t>
+  </si>
+  <si>
+    <t>690 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>922145316</t>
+  </si>
+  <si>
+    <t>956637958</t>
+  </si>
+  <si>
+    <t>enriquelopezruz@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>74833</t>
+  </si>
+  <si>
+    <t>4-K-25</t>
+  </si>
+  <si>
+    <t>1015721</t>
+  </si>
+  <si>
+    <t>11039322-9</t>
+  </si>
+  <si>
+    <t>CAYUN COÑOMAN ELIZARDO FREDDY</t>
+  </si>
+  <si>
+    <t>26/04/1965</t>
+  </si>
+  <si>
+    <t>936883092</t>
+  </si>
+  <si>
+    <t>936883092 - 95899950</t>
+  </si>
+  <si>
+    <t>jessicaz.carrasco45@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>1015722</t>
+  </si>
+  <si>
+    <t>8431496-k</t>
+  </si>
+  <si>
+    <t>FUENTES ARAYA BEATRIZ DE LAS MERCEDEZ</t>
+  </si>
+  <si>
+    <t>09/08/1956</t>
+  </si>
+  <si>
+    <t>Colina</t>
+  </si>
+  <si>
+    <t>104 - Colina - Chacabuco -CP</t>
+  </si>
+  <si>
+    <t>966723315</t>
+  </si>
+  <si>
+    <t>966723315 - 56966723315</t>
+  </si>
+  <si>
+    <t>beatrizfuentesaraya@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>27/02/2026</t>
+  </si>
+  <si>
+    <t>Veronica Cecilia Gonzalez Morales</t>
+  </si>
+  <si>
+    <t>1015724</t>
+  </si>
+  <si>
+    <t>5233612-0</t>
+  </si>
+  <si>
+    <t>ZÚÑIGA BAGINSKY ROBERTO</t>
+  </si>
+  <si>
+    <t>05/04/1944</t>
+  </si>
+  <si>
+    <t>Lo Prado</t>
+  </si>
+  <si>
+    <t>25 - Lo Prado - Santiago -CP</t>
+  </si>
+  <si>
+    <t>965951520</t>
+  </si>
+  <si>
+    <t>czuñigab44@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>Micaela Tais Vargas Castillo</t>
+  </si>
+  <si>
+    <t>2932500</t>
+  </si>
+  <si>
+    <t>293250</t>
+  </si>
+  <si>
+    <t>2639250</t>
+  </si>
+  <si>
+    <t>36656</t>
+  </si>
+  <si>
+    <t>Valle del Descanso</t>
+  </si>
+  <si>
+    <t>7-A-030</t>
+  </si>
+  <si>
+    <t>1015730</t>
+  </si>
+  <si>
+    <t>8045408-2</t>
+  </si>
+  <si>
+    <t>PEÑALOZA SANDOVAL ELBA ANGELA</t>
+  </si>
+  <si>
+    <t>15/03/1959</t>
+  </si>
+  <si>
+    <t>559 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>984167803</t>
+  </si>
+  <si>
+    <t>penaloza.elbas59@gmai.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>3220000</t>
+  </si>
+  <si>
+    <t>2705882.35</t>
+  </si>
+  <si>
+    <t>2705882</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>1015732</t>
+  </si>
+  <si>
+    <t>Valparaíso</t>
+  </si>
+  <si>
+    <t>7192742-3</t>
+  </si>
+  <si>
+    <t>RIOS ITURRA MARIO HUMBERTO</t>
+  </si>
+  <si>
+    <t>28/05/1955</t>
+  </si>
+  <si>
+    <t>San Antonio</t>
+  </si>
+  <si>
+    <t>890 - San Antonio - San Antonio -CP</t>
+  </si>
+  <si>
+    <t>987209124</t>
+  </si>
+  <si>
+    <t>proferios@hotmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>Katherine Andrea Romero Millan</t>
+  </si>
+  <si>
+    <t>4600000</t>
+  </si>
+  <si>
+    <t>3865546.22</t>
+  </si>
+  <si>
+    <t>3865546</t>
+  </si>
+  <si>
+    <t>172500</t>
+  </si>
+  <si>
+    <t>1015733</t>
+  </si>
+  <si>
+    <t>14355767-7</t>
+  </si>
+  <si>
+    <t>GÓMEZ URQUIOLA GABRIEL ALEJANDRO</t>
+  </si>
+  <si>
+    <t>20/07/1979</t>
+  </si>
+  <si>
+    <t>1919 - Lampa - Chacabuco -CP</t>
+  </si>
+  <si>
+    <t>934465509 - 56934465509</t>
+  </si>
+  <si>
+    <t>gomezurquiola@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>103500</t>
+  </si>
+  <si>
+    <t>1015734</t>
+  </si>
+  <si>
+    <t>12353329-1</t>
+  </si>
+  <si>
+    <t>ROBLES CISTERNAS MARGARITA ALEJANDRA</t>
+  </si>
+  <si>
+    <t>04/06/1973</t>
+  </si>
+  <si>
+    <t>358 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>994485350</t>
+  </si>
+  <si>
+    <t>robles.cisterm@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>Lidia Monica Flores Bravo</t>
+  </si>
+  <si>
+    <t>4490000</t>
+  </si>
+  <si>
+    <t>76102</t>
+  </si>
+  <si>
+    <t>3-V-21</t>
+  </si>
+  <si>
+    <t>1015735</t>
   </si>
 </sst>
 </file>
@@ -2257,7 +2572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP32"/>
+  <dimension ref="A1:AP42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="41" width="8" customWidth="1"/>
@@ -3758,7 +4073,7 @@
         <v>228</v>
       </c>
       <c r="AC12" t="s">
-        <v>185</v>
+        <v>67</v>
       </c>
       <c r="AD12" t="s">
         <v>68</v>
@@ -6358,6 +6673,1286 @@
       </c>
       <c r="AP32" t="s">
         <v>458</v>
+      </c>
+    </row>
+    <row r="33" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" t="s">
+        <v>459</v>
+      </c>
+      <c r="D33" t="s">
+        <v>460</v>
+      </c>
+      <c r="E33" t="s">
+        <v>461</v>
+      </c>
+      <c r="F33" t="s">
+        <v>327</v>
+      </c>
+      <c r="G33" t="s">
+        <v>462</v>
+      </c>
+      <c r="H33" t="s">
+        <v>463</v>
+      </c>
+      <c r="I33" t="s">
+        <v>464</v>
+      </c>
+      <c r="J33" t="s">
+        <v>465</v>
+      </c>
+      <c r="K33" t="s">
+        <v>319</v>
+      </c>
+      <c r="L33" t="s">
+        <v>381</v>
+      </c>
+      <c r="M33" t="s">
+        <v>86</v>
+      </c>
+      <c r="N33" t="s">
+        <v>55</v>
+      </c>
+      <c r="O33" t="s">
+        <v>87</v>
+      </c>
+      <c r="P33" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>138</v>
+      </c>
+      <c r="R33" t="s">
+        <v>90</v>
+      </c>
+      <c r="S33" t="s">
+        <v>91</v>
+      </c>
+      <c r="T33" t="s">
+        <v>92</v>
+      </c>
+      <c r="U33" t="s">
+        <v>60</v>
+      </c>
+      <c r="V33" t="s">
+        <v>60</v>
+      </c>
+      <c r="W33" t="s">
+        <v>93</v>
+      </c>
+      <c r="X33" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>345</v>
+      </c>
+      <c r="Z33" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA33" t="s">
+        <v>227</v>
+      </c>
+      <c r="AB33" t="s">
+        <v>261</v>
+      </c>
+      <c r="AC33" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD33" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE33" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF33" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG33" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH33" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI33" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ33" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK33" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL33" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM33" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN33" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO33" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP33" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="34" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" t="s">
+        <v>468</v>
+      </c>
+      <c r="D34" t="s">
+        <v>469</v>
+      </c>
+      <c r="E34" t="s">
+        <v>470</v>
+      </c>
+      <c r="F34" t="s">
+        <v>47</v>
+      </c>
+      <c r="G34" t="s">
+        <v>471</v>
+      </c>
+      <c r="H34" t="s">
+        <v>49</v>
+      </c>
+      <c r="I34" t="s">
+        <v>472</v>
+      </c>
+      <c r="J34" t="s">
+        <v>473</v>
+      </c>
+      <c r="K34" t="s">
+        <v>474</v>
+      </c>
+      <c r="L34" t="s">
+        <v>381</v>
+      </c>
+      <c r="M34" t="s">
+        <v>86</v>
+      </c>
+      <c r="N34" t="s">
+        <v>55</v>
+      </c>
+      <c r="O34" t="s">
+        <v>153</v>
+      </c>
+      <c r="P34" t="s">
+        <v>259</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>321</v>
+      </c>
+      <c r="R34" t="s">
+        <v>90</v>
+      </c>
+      <c r="S34" t="s">
+        <v>91</v>
+      </c>
+      <c r="T34" t="s">
+        <v>92</v>
+      </c>
+      <c r="U34" t="s">
+        <v>60</v>
+      </c>
+      <c r="V34" t="s">
+        <v>60</v>
+      </c>
+      <c r="W34" t="s">
+        <v>93</v>
+      </c>
+      <c r="X34" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y34" t="s">
+        <v>475</v>
+      </c>
+      <c r="Z34" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA34" t="s">
+        <v>96</v>
+      </c>
+      <c r="AB34" t="s">
+        <v>322</v>
+      </c>
+      <c r="AC34" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD34" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE34" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF34" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG34" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH34" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI34" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ34" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK34" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL34" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM34" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN34" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO34" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP34" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="35" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35" t="s">
+        <v>43</v>
+      </c>
+      <c r="C35" t="s">
+        <v>477</v>
+      </c>
+      <c r="D35" t="s">
+        <v>478</v>
+      </c>
+      <c r="E35" t="s">
+        <v>479</v>
+      </c>
+      <c r="F35" t="s">
+        <v>47</v>
+      </c>
+      <c r="G35" t="s">
+        <v>480</v>
+      </c>
+      <c r="H35" t="s">
+        <v>481</v>
+      </c>
+      <c r="I35" t="s">
+        <v>482</v>
+      </c>
+      <c r="J35" t="s">
+        <v>483</v>
+      </c>
+      <c r="K35" t="s">
+        <v>380</v>
+      </c>
+      <c r="L35" t="s">
+        <v>381</v>
+      </c>
+      <c r="M35" t="s">
+        <v>54</v>
+      </c>
+      <c r="N35" t="s">
+        <v>55</v>
+      </c>
+      <c r="O35" t="s">
+        <v>240</v>
+      </c>
+      <c r="P35" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>89</v>
+      </c>
+      <c r="R35" t="s">
+        <v>142</v>
+      </c>
+      <c r="S35" t="s">
+        <v>142</v>
+      </c>
+      <c r="T35" t="s">
+        <v>142</v>
+      </c>
+      <c r="U35" t="s">
+        <v>60</v>
+      </c>
+      <c r="V35" t="s">
+        <v>60</v>
+      </c>
+      <c r="W35" t="s">
+        <v>309</v>
+      </c>
+      <c r="X35" t="s">
+        <v>295</v>
+      </c>
+      <c r="Y35" t="s">
+        <v>381</v>
+      </c>
+      <c r="Z35" t="s">
+        <v>310</v>
+      </c>
+      <c r="AA35" t="s">
+        <v>371</v>
+      </c>
+      <c r="AB35" t="s">
+        <v>484</v>
+      </c>
+      <c r="AC35" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD35" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE35" t="s">
+        <v>172</v>
+      </c>
+      <c r="AF35" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG35" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH35" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI35" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ35" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK35" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL35" t="s">
+        <v>229</v>
+      </c>
+      <c r="AM35" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN35" t="s">
+        <v>416</v>
+      </c>
+      <c r="AO35" t="s">
+        <v>485</v>
+      </c>
+      <c r="AP35" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="36" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" t="s">
+        <v>43</v>
+      </c>
+      <c r="C36" t="s">
+        <v>487</v>
+      </c>
+      <c r="D36" t="s">
+        <v>488</v>
+      </c>
+      <c r="E36" t="s">
+        <v>489</v>
+      </c>
+      <c r="F36" t="s">
+        <v>327</v>
+      </c>
+      <c r="G36" t="s">
+        <v>462</v>
+      </c>
+      <c r="H36" t="s">
+        <v>490</v>
+      </c>
+      <c r="I36" t="s">
+        <v>491</v>
+      </c>
+      <c r="J36" t="s">
+        <v>492</v>
+      </c>
+      <c r="K36" t="s">
+        <v>319</v>
+      </c>
+      <c r="L36" t="s">
+        <v>381</v>
+      </c>
+      <c r="M36" t="s">
+        <v>86</v>
+      </c>
+      <c r="N36" t="s">
+        <v>55</v>
+      </c>
+      <c r="O36" t="s">
+        <v>87</v>
+      </c>
+      <c r="P36" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>138</v>
+      </c>
+      <c r="R36" t="s">
+        <v>90</v>
+      </c>
+      <c r="S36" t="s">
+        <v>91</v>
+      </c>
+      <c r="T36" t="s">
+        <v>92</v>
+      </c>
+      <c r="U36" t="s">
+        <v>60</v>
+      </c>
+      <c r="V36" t="s">
+        <v>60</v>
+      </c>
+      <c r="W36" t="s">
+        <v>93</v>
+      </c>
+      <c r="X36" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y36" t="s">
+        <v>475</v>
+      </c>
+      <c r="Z36" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA36" t="s">
+        <v>227</v>
+      </c>
+      <c r="AB36" t="s">
+        <v>261</v>
+      </c>
+      <c r="AC36" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD36" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE36" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF36" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG36" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH36" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI36" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ36" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK36" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL36" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM36" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN36" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO36" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP36" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="37" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37" t="s">
+        <v>43</v>
+      </c>
+      <c r="C37" t="s">
+        <v>494</v>
+      </c>
+      <c r="D37" t="s">
+        <v>495</v>
+      </c>
+      <c r="E37" t="s">
+        <v>496</v>
+      </c>
+      <c r="F37" t="s">
+        <v>497</v>
+      </c>
+      <c r="G37" t="s">
+        <v>498</v>
+      </c>
+      <c r="H37" t="s">
+        <v>499</v>
+      </c>
+      <c r="I37" t="s">
+        <v>500</v>
+      </c>
+      <c r="J37" t="s">
+        <v>501</v>
+      </c>
+      <c r="K37" t="s">
+        <v>502</v>
+      </c>
+      <c r="L37" t="s">
+        <v>381</v>
+      </c>
+      <c r="M37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N37" t="s">
+        <v>55</v>
+      </c>
+      <c r="O37" t="s">
+        <v>240</v>
+      </c>
+      <c r="P37" t="s">
+        <v>503</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>89</v>
+      </c>
+      <c r="R37" t="s">
+        <v>90</v>
+      </c>
+      <c r="S37" t="s">
+        <v>91</v>
+      </c>
+      <c r="T37" t="s">
+        <v>92</v>
+      </c>
+      <c r="U37" t="s">
+        <v>60</v>
+      </c>
+      <c r="V37" t="s">
+        <v>60</v>
+      </c>
+      <c r="W37" t="s">
+        <v>93</v>
+      </c>
+      <c r="X37" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y37" t="s">
+        <v>475</v>
+      </c>
+      <c r="Z37" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA37" t="s">
+        <v>227</v>
+      </c>
+      <c r="AB37" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC37" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD37" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE37" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF37" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG37" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH37" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI37" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ37" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK37" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL37" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM37" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN37" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO37" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP37" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="38" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C38" t="s">
+        <v>505</v>
+      </c>
+      <c r="D38" t="s">
+        <v>506</v>
+      </c>
+      <c r="E38" t="s">
+        <v>507</v>
+      </c>
+      <c r="F38" t="s">
+        <v>508</v>
+      </c>
+      <c r="G38" t="s">
+        <v>509</v>
+      </c>
+      <c r="H38" t="s">
+        <v>49</v>
+      </c>
+      <c r="I38" t="s">
+        <v>510</v>
+      </c>
+      <c r="J38" t="s">
+        <v>511</v>
+      </c>
+      <c r="K38" t="s">
+        <v>135</v>
+      </c>
+      <c r="L38" t="s">
+        <v>381</v>
+      </c>
+      <c r="M38" t="s">
+        <v>54</v>
+      </c>
+      <c r="N38" t="s">
+        <v>55</v>
+      </c>
+      <c r="O38" t="s">
+        <v>87</v>
+      </c>
+      <c r="P38" t="s">
+        <v>512</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>58</v>
+      </c>
+      <c r="R38" t="s">
+        <v>513</v>
+      </c>
+      <c r="S38" t="s">
+        <v>513</v>
+      </c>
+      <c r="T38" t="s">
+        <v>513</v>
+      </c>
+      <c r="U38" t="s">
+        <v>60</v>
+      </c>
+      <c r="V38" t="s">
+        <v>60</v>
+      </c>
+      <c r="W38" t="s">
+        <v>93</v>
+      </c>
+      <c r="X38" t="s">
+        <v>514</v>
+      </c>
+      <c r="Y38" t="s">
+        <v>410</v>
+      </c>
+      <c r="Z38" t="s">
+        <v>515</v>
+      </c>
+      <c r="AA38" t="s">
+        <v>227</v>
+      </c>
+      <c r="AB38" t="s">
+        <v>516</v>
+      </c>
+      <c r="AC38" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD38" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE38" t="s">
+        <v>299</v>
+      </c>
+      <c r="AF38" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG38" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH38" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI38" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ38" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK38" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL38" t="s">
+        <v>517</v>
+      </c>
+      <c r="AM38" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN38" t="s">
+        <v>73</v>
+      </c>
+      <c r="AO38" t="s">
+        <v>518</v>
+      </c>
+      <c r="AP38" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="39" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" t="s">
+        <v>43</v>
+      </c>
+      <c r="C39" t="s">
+        <v>520</v>
+      </c>
+      <c r="D39" t="s">
+        <v>521</v>
+      </c>
+      <c r="E39" t="s">
+        <v>522</v>
+      </c>
+      <c r="F39" t="s">
+        <v>47</v>
+      </c>
+      <c r="G39" t="s">
+        <v>523</v>
+      </c>
+      <c r="H39" t="s">
+        <v>524</v>
+      </c>
+      <c r="I39" t="s">
+        <v>524</v>
+      </c>
+      <c r="J39" t="s">
+        <v>525</v>
+      </c>
+      <c r="K39" t="s">
+        <v>385</v>
+      </c>
+      <c r="L39" t="s">
+        <v>381</v>
+      </c>
+      <c r="M39" t="s">
+        <v>120</v>
+      </c>
+      <c r="N39" t="s">
+        <v>55</v>
+      </c>
+      <c r="O39" t="s">
+        <v>87</v>
+      </c>
+      <c r="P39" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>60</v>
+      </c>
+      <c r="R39" t="s">
+        <v>526</v>
+      </c>
+      <c r="S39" t="s">
+        <v>527</v>
+      </c>
+      <c r="T39" t="s">
+        <v>528</v>
+      </c>
+      <c r="U39" t="s">
+        <v>60</v>
+      </c>
+      <c r="V39" t="s">
+        <v>60</v>
+      </c>
+      <c r="W39" t="s">
+        <v>529</v>
+      </c>
+      <c r="X39" t="s">
+        <v>526</v>
+      </c>
+      <c r="Y39" t="s">
+        <v>385</v>
+      </c>
+      <c r="Z39" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA39" t="s">
+        <v>65</v>
+      </c>
+      <c r="AB39" t="s">
+        <v>526</v>
+      </c>
+      <c r="AC39" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD39" t="s">
+        <v>127</v>
+      </c>
+      <c r="AE39" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF39" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG39" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH39" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI39" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ39" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK39" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL39" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM39" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN39" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO39" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP39" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="40" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" t="s">
+        <v>531</v>
+      </c>
+      <c r="C40" t="s">
+        <v>532</v>
+      </c>
+      <c r="D40" t="s">
+        <v>533</v>
+      </c>
+      <c r="E40" t="s">
+        <v>534</v>
+      </c>
+      <c r="F40" t="s">
+        <v>535</v>
+      </c>
+      <c r="G40" t="s">
+        <v>536</v>
+      </c>
+      <c r="H40" t="s">
+        <v>537</v>
+      </c>
+      <c r="I40" t="s">
+        <v>537</v>
+      </c>
+      <c r="J40" t="s">
+        <v>538</v>
+      </c>
+      <c r="K40" t="s">
+        <v>410</v>
+      </c>
+      <c r="L40" t="s">
+        <v>381</v>
+      </c>
+      <c r="M40" t="s">
+        <v>120</v>
+      </c>
+      <c r="N40" t="s">
+        <v>55</v>
+      </c>
+      <c r="O40" t="s">
+        <v>153</v>
+      </c>
+      <c r="P40" t="s">
+        <v>539</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>359</v>
+      </c>
+      <c r="R40" t="s">
+        <v>540</v>
+      </c>
+      <c r="S40" t="s">
+        <v>541</v>
+      </c>
+      <c r="T40" t="s">
+        <v>542</v>
+      </c>
+      <c r="U40" t="s">
+        <v>60</v>
+      </c>
+      <c r="V40" t="s">
+        <v>60</v>
+      </c>
+      <c r="W40" t="s">
+        <v>93</v>
+      </c>
+      <c r="X40" t="s">
+        <v>155</v>
+      </c>
+      <c r="Y40" t="s">
+        <v>381</v>
+      </c>
+      <c r="Z40" t="s">
+        <v>121</v>
+      </c>
+      <c r="AA40" t="s">
+        <v>391</v>
+      </c>
+      <c r="AB40" t="s">
+        <v>543</v>
+      </c>
+      <c r="AC40" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD40" t="s">
+        <v>127</v>
+      </c>
+      <c r="AE40" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF40" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG40" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH40" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI40" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ40" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK40" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL40" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM40" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN40" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO40" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP40" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="41" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" t="s">
+        <v>43</v>
+      </c>
+      <c r="C41" t="s">
+        <v>545</v>
+      </c>
+      <c r="D41" t="s">
+        <v>546</v>
+      </c>
+      <c r="E41" t="s">
+        <v>547</v>
+      </c>
+      <c r="F41" t="s">
+        <v>103</v>
+      </c>
+      <c r="G41" t="s">
+        <v>548</v>
+      </c>
+      <c r="H41" t="s">
+        <v>49</v>
+      </c>
+      <c r="I41" t="s">
+        <v>549</v>
+      </c>
+      <c r="J41" t="s">
+        <v>550</v>
+      </c>
+      <c r="K41" t="s">
+        <v>53</v>
+      </c>
+      <c r="L41" t="s">
+        <v>381</v>
+      </c>
+      <c r="M41" t="s">
+        <v>120</v>
+      </c>
+      <c r="N41" t="s">
+        <v>55</v>
+      </c>
+      <c r="O41" t="s">
+        <v>240</v>
+      </c>
+      <c r="P41" t="s">
+        <v>503</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>199</v>
+      </c>
+      <c r="R41" t="s">
+        <v>121</v>
+      </c>
+      <c r="S41" t="s">
+        <v>122</v>
+      </c>
+      <c r="T41" t="s">
+        <v>123</v>
+      </c>
+      <c r="U41" t="s">
+        <v>60</v>
+      </c>
+      <c r="V41" t="s">
+        <v>60</v>
+      </c>
+      <c r="W41" t="s">
+        <v>93</v>
+      </c>
+      <c r="X41" t="s">
+        <v>124</v>
+      </c>
+      <c r="Y41" t="s">
+        <v>381</v>
+      </c>
+      <c r="Z41" t="s">
+        <v>125</v>
+      </c>
+      <c r="AA41" t="s">
+        <v>227</v>
+      </c>
+      <c r="AB41" t="s">
+        <v>551</v>
+      </c>
+      <c r="AC41" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD41" t="s">
+        <v>127</v>
+      </c>
+      <c r="AE41" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF41" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG41" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH41" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI41" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ41" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK41" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL41" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM41" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN41" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO41" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP41" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="42" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42" t="s">
+        <v>43</v>
+      </c>
+      <c r="C42" t="s">
+        <v>553</v>
+      </c>
+      <c r="D42" t="s">
+        <v>554</v>
+      </c>
+      <c r="E42" t="s">
+        <v>555</v>
+      </c>
+      <c r="F42" t="s">
+        <v>47</v>
+      </c>
+      <c r="G42" t="s">
+        <v>556</v>
+      </c>
+      <c r="H42" t="s">
+        <v>49</v>
+      </c>
+      <c r="I42" t="s">
+        <v>557</v>
+      </c>
+      <c r="J42" t="s">
+        <v>558</v>
+      </c>
+      <c r="K42" t="s">
+        <v>381</v>
+      </c>
+      <c r="L42" t="s">
+        <v>381</v>
+      </c>
+      <c r="M42" t="s">
+        <v>54</v>
+      </c>
+      <c r="N42" t="s">
+        <v>55</v>
+      </c>
+      <c r="O42" t="s">
+        <v>153</v>
+      </c>
+      <c r="P42" t="s">
+        <v>559</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>321</v>
+      </c>
+      <c r="R42" t="s">
+        <v>59</v>
+      </c>
+      <c r="S42" t="s">
+        <v>59</v>
+      </c>
+      <c r="T42" t="s">
+        <v>59</v>
+      </c>
+      <c r="U42" t="s">
+        <v>60</v>
+      </c>
+      <c r="V42" t="s">
+        <v>60</v>
+      </c>
+      <c r="W42" t="s">
+        <v>309</v>
+      </c>
+      <c r="X42" t="s">
+        <v>454</v>
+      </c>
+      <c r="Y42" t="s">
+        <v>475</v>
+      </c>
+      <c r="Z42" t="s">
+        <v>560</v>
+      </c>
+      <c r="AA42" t="s">
+        <v>227</v>
+      </c>
+      <c r="AB42" t="s">
+        <v>561</v>
+      </c>
+      <c r="AC42" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD42" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE42" t="s">
+        <v>172</v>
+      </c>
+      <c r="AF42" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG42" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH42" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI42" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ42" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK42" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL42" t="s">
+        <v>173</v>
+      </c>
+      <c r="AM42" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN42" t="s">
+        <v>73</v>
+      </c>
+      <c r="AO42" t="s">
+        <v>562</v>
+      </c>
+      <c r="AP42" t="s">
+        <v>563</v>
       </c>
     </row>
   </sheetData>

</xml_diff>